<commit_message>
July 2, 2026 deck v3 — VR peerset exactness (member-for-member vs BirlaMFPR) + category reconciliation (0-bucket dissolved: VR/SEBI categories; VR peers immune to All-Peers exclusions)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/July 2, 2026/Data/Mapping/Map MFI Scheme to Category.xlsx
+++ b/July 2, 2026/Data/Mapping/Map MFI Scheme to Category.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H951"/>
+  <dimension ref="A1:H954"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Thematic</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Thematic</t>
+          <t>Business Cycle</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Thematic</t>
+          <t>Business Cycle</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -4861,7 +4861,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Thematic</t>
+          <t>Business Cycle</t>
         </is>
       </c>
       <c r="F117" t="n">
@@ -9003,7 +9003,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Thematic</t>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="F226" t="n">
@@ -10485,7 +10485,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Thematic</t>
+          <t>MNC</t>
         </is>
       </c>
       <c r="F265" t="n">
@@ -12157,7 +12157,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Thematic</t>
+          <t>Business Cycle</t>
         </is>
       </c>
       <c r="F309" t="n">
@@ -12499,7 +12499,7 @@
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>Thematic</t>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="F318" t="n">
@@ -15159,7 +15159,7 @@
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t>Thematic</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F388" t="n">
@@ -15843,7 +15843,7 @@
       </c>
       <c r="E406" t="inlineStr">
         <is>
-          <t>Sectoral</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="F406" t="n">
@@ -15957,7 +15957,7 @@
       </c>
       <c r="E409" t="inlineStr">
         <is>
-          <t>Thematic</t>
+          <t>Business Cycle</t>
         </is>
       </c>
       <c r="F409" t="n">
@@ -15995,7 +15995,7 @@
       </c>
       <c r="E410" t="inlineStr">
         <is>
-          <t>consumption</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F410" t="n">
@@ -27315,8 +27315,10 @@
       <c r="D708" t="n">
         <v>0</v>
       </c>
-      <c r="E708" t="n">
-        <v>0</v>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F708" t="n">
         <v>0</v>
@@ -27349,8 +27351,10 @@
       <c r="D709" t="n">
         <v>0</v>
       </c>
-      <c r="E709" t="n">
-        <v>0</v>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F709" t="n">
         <v>0</v>
@@ -27383,8 +27387,10 @@
       <c r="D710" t="n">
         <v>0</v>
       </c>
-      <c r="E710" t="n">
-        <v>0</v>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F710" t="n">
         <v>0</v>
@@ -27417,8 +27423,10 @@
       <c r="D711" t="n">
         <v>0</v>
       </c>
-      <c r="E711" t="n">
-        <v>0</v>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F711" t="n">
         <v>0</v>
@@ -27451,8 +27459,10 @@
       <c r="D712" t="n">
         <v>0</v>
       </c>
-      <c r="E712" t="n">
-        <v>0</v>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F712" t="n">
         <v>0</v>
@@ -27485,8 +27495,10 @@
       <c r="D713" t="n">
         <v>0</v>
       </c>
-      <c r="E713" t="n">
-        <v>0</v>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F713" t="n">
         <v>0</v>
@@ -27519,8 +27531,10 @@
       <c r="D714" t="n">
         <v>0</v>
       </c>
-      <c r="E714" t="n">
-        <v>0</v>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F714" t="n">
         <v>0</v>
@@ -27553,8 +27567,10 @@
       <c r="D715" t="n">
         <v>0</v>
       </c>
-      <c r="E715" t="n">
-        <v>0</v>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>Multi Index FoF</t>
+        </is>
       </c>
       <c r="F715" t="n">
         <v>0</v>
@@ -27587,8 +27603,10 @@
       <c r="D716" t="n">
         <v>0</v>
       </c>
-      <c r="E716" t="n">
-        <v>0</v>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>Asset Allocator Funds</t>
+        </is>
       </c>
       <c r="F716" t="n">
         <v>0</v>
@@ -27621,8 +27639,10 @@
       <c r="D717" t="n">
         <v>0</v>
       </c>
-      <c r="E717" t="n">
-        <v>0</v>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>Silver FoF</t>
+        </is>
       </c>
       <c r="F717" t="n">
         <v>0</v>
@@ -27655,8 +27675,10 @@
       <c r="D718" t="n">
         <v>0</v>
       </c>
-      <c r="E718" t="n">
-        <v>0</v>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F718" t="n">
         <v>0</v>
@@ -27689,8 +27711,10 @@
       <c r="D719" t="n">
         <v>0</v>
       </c>
-      <c r="E719" t="n">
-        <v>0</v>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F719" t="n">
         <v>0</v>
@@ -27723,8 +27747,10 @@
       <c r="D720" t="n">
         <v>0</v>
       </c>
-      <c r="E720" t="n">
-        <v>0</v>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F720" t="n">
         <v>0</v>
@@ -27757,8 +27783,10 @@
       <c r="D721" t="n">
         <v>0</v>
       </c>
-      <c r="E721" t="n">
-        <v>0</v>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F721" t="n">
         <v>0</v>
@@ -27791,8 +27819,10 @@
       <c r="D722" t="n">
         <v>0</v>
       </c>
-      <c r="E722" t="n">
-        <v>0</v>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F722" t="n">
         <v>0</v>
@@ -27825,8 +27855,10 @@
       <c r="D723" t="n">
         <v>0</v>
       </c>
-      <c r="E723" t="n">
-        <v>0</v>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F723" t="n">
         <v>0</v>
@@ -27859,8 +27891,10 @@
       <c r="D724" t="n">
         <v>0</v>
       </c>
-      <c r="E724" t="n">
-        <v>0</v>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F724" t="n">
         <v>0</v>
@@ -27893,8 +27927,10 @@
       <c r="D725" t="n">
         <v>0</v>
       </c>
-      <c r="E725" t="n">
-        <v>0</v>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F725" t="n">
         <v>0</v>
@@ -27927,8 +27963,10 @@
       <c r="D726" t="n">
         <v>0</v>
       </c>
-      <c r="E726" t="n">
-        <v>0</v>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F726" t="n">
         <v>0</v>
@@ -27961,8 +27999,10 @@
       <c r="D727" t="n">
         <v>0</v>
       </c>
-      <c r="E727" t="n">
-        <v>0</v>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>Silver FoF</t>
+        </is>
       </c>
       <c r="F727" t="n">
         <v>0</v>
@@ -27995,8 +28035,10 @@
       <c r="D728" t="n">
         <v>0</v>
       </c>
-      <c r="E728" t="n">
-        <v>0</v>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>Asset Allocator Funds</t>
+        </is>
       </c>
       <c r="F728" t="n">
         <v>0</v>
@@ -28029,8 +28071,10 @@
       <c r="D729" t="n">
         <v>0</v>
       </c>
-      <c r="E729" t="n">
-        <v>0</v>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>Asset Allocator Funds</t>
+        </is>
       </c>
       <c r="F729" t="n">
         <v>0</v>
@@ -28063,8 +28107,10 @@
       <c r="D730" t="n">
         <v>0</v>
       </c>
-      <c r="E730" t="n">
-        <v>0</v>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F730" t="n">
         <v>0</v>
@@ -28097,8 +28143,10 @@
       <c r="D731" t="n">
         <v>0</v>
       </c>
-      <c r="E731" t="n">
-        <v>0</v>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>Asset Allocator Funds</t>
+        </is>
       </c>
       <c r="F731" t="n">
         <v>0</v>
@@ -28131,8 +28179,10 @@
       <c r="D732" t="n">
         <v>0</v>
       </c>
-      <c r="E732" t="n">
-        <v>0</v>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F732" t="n">
         <v>0</v>
@@ -28165,8 +28215,10 @@
       <c r="D733" t="n">
         <v>0</v>
       </c>
-      <c r="E733" t="n">
-        <v>0</v>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F733" t="n">
         <v>0</v>
@@ -28199,8 +28251,10 @@
       <c r="D734" t="n">
         <v>0</v>
       </c>
-      <c r="E734" t="n">
-        <v>0</v>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F734" t="n">
         <v>0</v>
@@ -28233,8 +28287,10 @@
       <c r="D735" t="n">
         <v>0</v>
       </c>
-      <c r="E735" t="n">
-        <v>0</v>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F735" t="n">
         <v>0</v>
@@ -28267,8 +28323,10 @@
       <c r="D736" t="n">
         <v>0</v>
       </c>
-      <c r="E736" t="n">
-        <v>0</v>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F736" t="n">
         <v>0</v>
@@ -28301,8 +28359,10 @@
       <c r="D737" t="n">
         <v>0</v>
       </c>
-      <c r="E737" t="n">
-        <v>0</v>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F737" t="n">
         <v>0</v>
@@ -28335,8 +28395,10 @@
       <c r="D738" t="n">
         <v>0</v>
       </c>
-      <c r="E738" t="n">
-        <v>0</v>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F738" t="n">
         <v>0</v>
@@ -28369,8 +28431,10 @@
       <c r="D739" t="n">
         <v>0</v>
       </c>
-      <c r="E739" t="n">
-        <v>0</v>
+      <c r="E739" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F739" t="n">
         <v>0</v>
@@ -28403,8 +28467,10 @@
       <c r="D740" t="n">
         <v>0</v>
       </c>
-      <c r="E740" t="n">
-        <v>0</v>
+      <c r="E740" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F740" t="n">
         <v>0</v>
@@ -28437,8 +28503,10 @@
       <c r="D741" t="n">
         <v>0</v>
       </c>
-      <c r="E741" t="n">
-        <v>0</v>
+      <c r="E741" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F741" t="n">
         <v>0</v>
@@ -28471,8 +28539,10 @@
       <c r="D742" t="n">
         <v>0</v>
       </c>
-      <c r="E742" t="n">
-        <v>0</v>
+      <c r="E742" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F742" t="n">
         <v>0</v>
@@ -28505,8 +28575,10 @@
       <c r="D743" t="n">
         <v>0</v>
       </c>
-      <c r="E743" t="n">
-        <v>0</v>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F743" t="n">
         <v>0</v>
@@ -28539,8 +28611,10 @@
       <c r="D744" t="n">
         <v>0</v>
       </c>
-      <c r="E744" t="n">
-        <v>0</v>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F744" t="n">
         <v>0</v>
@@ -28573,8 +28647,10 @@
       <c r="D745" t="n">
         <v>0</v>
       </c>
-      <c r="E745" t="n">
-        <v>0</v>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F745" t="n">
         <v>0</v>
@@ -28607,8 +28683,10 @@
       <c r="D746" t="n">
         <v>0</v>
       </c>
-      <c r="E746" t="n">
-        <v>0</v>
+      <c r="E746" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F746" t="n">
         <v>0</v>
@@ -28641,8 +28719,10 @@
       <c r="D747" t="n">
         <v>0</v>
       </c>
-      <c r="E747" t="n">
-        <v>0</v>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F747" t="n">
         <v>0</v>
@@ -28675,8 +28755,10 @@
       <c r="D748" t="n">
         <v>0</v>
       </c>
-      <c r="E748" t="n">
-        <v>0</v>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F748" t="n">
         <v>0</v>
@@ -28709,8 +28791,10 @@
       <c r="D749" t="n">
         <v>0</v>
       </c>
-      <c r="E749" t="n">
-        <v>0</v>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F749" t="n">
         <v>0</v>
@@ -28743,8 +28827,10 @@
       <c r="D750" t="n">
         <v>0</v>
       </c>
-      <c r="E750" t="n">
-        <v>0</v>
+      <c r="E750" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F750" t="n">
         <v>0</v>
@@ -28777,8 +28863,10 @@
       <c r="D751" t="n">
         <v>0</v>
       </c>
-      <c r="E751" t="n">
-        <v>0</v>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F751" t="n">
         <v>0</v>
@@ -28811,8 +28899,10 @@
       <c r="D752" t="n">
         <v>0</v>
       </c>
-      <c r="E752" t="n">
-        <v>0</v>
+      <c r="E752" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F752" t="n">
         <v>0</v>
@@ -28845,8 +28935,10 @@
       <c r="D753" t="n">
         <v>0</v>
       </c>
-      <c r="E753" t="n">
-        <v>0</v>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F753" t="n">
         <v>0</v>
@@ -28879,8 +28971,10 @@
       <c r="D754" t="n">
         <v>0</v>
       </c>
-      <c r="E754" t="n">
-        <v>0</v>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F754" t="n">
         <v>0</v>
@@ -28913,8 +29007,10 @@
       <c r="D755" t="n">
         <v>0</v>
       </c>
-      <c r="E755" t="n">
-        <v>0</v>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F755" t="n">
         <v>0</v>
@@ -28947,8 +29043,10 @@
       <c r="D756" t="n">
         <v>0</v>
       </c>
-      <c r="E756" t="n">
-        <v>0</v>
+      <c r="E756" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F756" t="n">
         <v>0</v>
@@ -28981,8 +29079,10 @@
       <c r="D757" t="n">
         <v>0</v>
       </c>
-      <c r="E757" t="n">
-        <v>0</v>
+      <c r="E757" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F757" t="n">
         <v>0</v>
@@ -29015,8 +29115,10 @@
       <c r="D758" t="n">
         <v>0</v>
       </c>
-      <c r="E758" t="n">
-        <v>0</v>
+      <c r="E758" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F758" t="n">
         <v>0</v>
@@ -29049,8 +29151,10 @@
       <c r="D759" t="n">
         <v>0</v>
       </c>
-      <c r="E759" t="n">
-        <v>0</v>
+      <c r="E759" t="inlineStr">
+        <is>
+          <t>Asset Allocator Funds</t>
+        </is>
       </c>
       <c r="F759" t="n">
         <v>0</v>
@@ -29083,8 +29187,10 @@
       <c r="D760" t="n">
         <v>0</v>
       </c>
-      <c r="E760" t="n">
-        <v>0</v>
+      <c r="E760" t="inlineStr">
+        <is>
+          <t>Asset Allocator Funds</t>
+        </is>
       </c>
       <c r="F760" t="n">
         <v>0</v>
@@ -29117,8 +29223,10 @@
       <c r="D761" t="n">
         <v>0</v>
       </c>
-      <c r="E761" t="n">
-        <v>0</v>
+      <c r="E761" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F761" t="n">
         <v>0</v>
@@ -29151,8 +29259,10 @@
       <c r="D762" t="n">
         <v>0</v>
       </c>
-      <c r="E762" t="n">
-        <v>0</v>
+      <c r="E762" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F762" t="n">
         <v>0</v>
@@ -29185,8 +29295,10 @@
       <c r="D763" t="n">
         <v>0</v>
       </c>
-      <c r="E763" t="n">
-        <v>0</v>
+      <c r="E763" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F763" t="n">
         <v>0</v>
@@ -29219,8 +29331,10 @@
       <c r="D764" t="n">
         <v>0</v>
       </c>
-      <c r="E764" t="n">
-        <v>0</v>
+      <c r="E764" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F764" t="n">
         <v>0</v>
@@ -29277,8 +29391,10 @@
       <c r="D766" t="n">
         <v>0</v>
       </c>
-      <c r="E766" t="n">
-        <v>0</v>
+      <c r="E766" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F766" t="n">
         <v>0</v>
@@ -29311,8 +29427,10 @@
       <c r="D767" t="n">
         <v>0</v>
       </c>
-      <c r="E767" t="n">
-        <v>0</v>
+      <c r="E767" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F767" t="n">
         <v>0</v>
@@ -29345,8 +29463,10 @@
       <c r="D768" t="n">
         <v>0</v>
       </c>
-      <c r="E768" t="n">
-        <v>0</v>
+      <c r="E768" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F768" t="n">
         <v>0</v>
@@ -29379,8 +29499,10 @@
       <c r="D769" t="n">
         <v>0</v>
       </c>
-      <c r="E769" t="n">
-        <v>0</v>
+      <c r="E769" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F769" t="n">
         <v>0</v>
@@ -29413,8 +29535,10 @@
       <c r="D770" t="n">
         <v>0</v>
       </c>
-      <c r="E770" t="n">
-        <v>0</v>
+      <c r="E770" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F770" t="n">
         <v>0</v>
@@ -29447,8 +29571,10 @@
       <c r="D771" t="n">
         <v>0</v>
       </c>
-      <c r="E771" t="n">
-        <v>0</v>
+      <c r="E771" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F771" t="n">
         <v>0</v>
@@ -29481,8 +29607,10 @@
       <c r="D772" t="n">
         <v>0</v>
       </c>
-      <c r="E772" t="n">
-        <v>0</v>
+      <c r="E772" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F772" t="n">
         <v>0</v>
@@ -29515,8 +29643,10 @@
       <c r="D773" t="n">
         <v>0</v>
       </c>
-      <c r="E773" t="n">
-        <v>0</v>
+      <c r="E773" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F773" t="n">
         <v>0</v>
@@ -29549,8 +29679,10 @@
       <c r="D774" t="n">
         <v>0</v>
       </c>
-      <c r="E774" t="n">
-        <v>0</v>
+      <c r="E774" t="inlineStr">
+        <is>
+          <t>Asset Allocator Funds</t>
+        </is>
       </c>
       <c r="F774" t="n">
         <v>0</v>
@@ -29583,8 +29715,10 @@
       <c r="D775" t="n">
         <v>0</v>
       </c>
-      <c r="E775" t="n">
-        <v>0</v>
+      <c r="E775" t="inlineStr">
+        <is>
+          <t>Silver FoF</t>
+        </is>
       </c>
       <c r="F775" t="n">
         <v>0</v>
@@ -29617,8 +29751,10 @@
       <c r="D776" t="n">
         <v>0</v>
       </c>
-      <c r="E776" t="n">
-        <v>0</v>
+      <c r="E776" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F776" t="n">
         <v>0</v>
@@ -29651,8 +29787,10 @@
       <c r="D777" t="n">
         <v>0</v>
       </c>
-      <c r="E777" t="n">
-        <v>0</v>
+      <c r="E777" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F777" t="n">
         <v>0</v>
@@ -29685,8 +29823,10 @@
       <c r="D778" t="n">
         <v>0</v>
       </c>
-      <c r="E778" t="n">
-        <v>0</v>
+      <c r="E778" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F778" t="n">
         <v>0</v>
@@ -29719,8 +29859,10 @@
       <c r="D779" t="n">
         <v>0</v>
       </c>
-      <c r="E779" t="n">
-        <v>0</v>
+      <c r="E779" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F779" t="n">
         <v>0</v>
@@ -29753,8 +29895,10 @@
       <c r="D780" t="n">
         <v>0</v>
       </c>
-      <c r="E780" t="n">
-        <v>0</v>
+      <c r="E780" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F780" t="n">
         <v>0</v>
@@ -29787,8 +29931,10 @@
       <c r="D781" t="n">
         <v>0</v>
       </c>
-      <c r="E781" t="n">
-        <v>0</v>
+      <c r="E781" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F781" t="n">
         <v>0</v>
@@ -29821,8 +29967,10 @@
       <c r="D782" t="n">
         <v>0</v>
       </c>
-      <c r="E782" t="n">
-        <v>0</v>
+      <c r="E782" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F782" t="n">
         <v>0</v>
@@ -29855,8 +30003,10 @@
       <c r="D783" t="n">
         <v>0</v>
       </c>
-      <c r="E783" t="n">
-        <v>0</v>
+      <c r="E783" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F783" t="n">
         <v>0</v>
@@ -29889,8 +30039,10 @@
       <c r="D784" t="n">
         <v>0</v>
       </c>
-      <c r="E784" t="n">
-        <v>0</v>
+      <c r="E784" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F784" t="n">
         <v>0</v>
@@ -29923,8 +30075,10 @@
       <c r="D785" t="n">
         <v>0</v>
       </c>
-      <c r="E785" t="n">
-        <v>0</v>
+      <c r="E785" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F785" t="n">
         <v>0</v>
@@ -29957,8 +30111,10 @@
       <c r="D786" t="n">
         <v>0</v>
       </c>
-      <c r="E786" t="n">
-        <v>0</v>
+      <c r="E786" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F786" t="n">
         <v>0</v>
@@ -29991,8 +30147,10 @@
       <c r="D787" t="n">
         <v>0</v>
       </c>
-      <c r="E787" t="n">
-        <v>0</v>
+      <c r="E787" t="inlineStr">
+        <is>
+          <t>Asset Allocator Funds</t>
+        </is>
       </c>
       <c r="F787" t="n">
         <v>0</v>
@@ -30025,8 +30183,10 @@
       <c r="D788" t="n">
         <v>0</v>
       </c>
-      <c r="E788" t="n">
-        <v>0</v>
+      <c r="E788" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F788" t="n">
         <v>0</v>
@@ -30059,8 +30219,10 @@
       <c r="D789" t="n">
         <v>0</v>
       </c>
-      <c r="E789" t="n">
-        <v>0</v>
+      <c r="E789" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F789" t="n">
         <v>0</v>
@@ -30093,8 +30255,10 @@
       <c r="D790" t="n">
         <v>0</v>
       </c>
-      <c r="E790" t="n">
-        <v>0</v>
+      <c r="E790" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F790" t="n">
         <v>0</v>
@@ -30127,8 +30291,10 @@
       <c r="D791" t="n">
         <v>0</v>
       </c>
-      <c r="E791" t="n">
-        <v>0</v>
+      <c r="E791" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F791" t="n">
         <v>0</v>
@@ -30161,8 +30327,10 @@
       <c r="D792" t="n">
         <v>0</v>
       </c>
-      <c r="E792" t="n">
-        <v>0</v>
+      <c r="E792" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F792" t="n">
         <v>0</v>
@@ -30195,8 +30363,10 @@
       <c r="D793" t="n">
         <v>0</v>
       </c>
-      <c r="E793" t="n">
-        <v>0</v>
+      <c r="E793" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F793" t="n">
         <v>0</v>
@@ -30229,8 +30399,10 @@
       <c r="D794" t="n">
         <v>0</v>
       </c>
-      <c r="E794" t="n">
-        <v>0</v>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F794" t="n">
         <v>0</v>
@@ -30263,8 +30435,10 @@
       <c r="D795" t="n">
         <v>0</v>
       </c>
-      <c r="E795" t="n">
-        <v>0</v>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F795" t="n">
         <v>0</v>
@@ -30297,8 +30471,10 @@
       <c r="D796" t="n">
         <v>0</v>
       </c>
-      <c r="E796" t="n">
-        <v>0</v>
+      <c r="E796" t="inlineStr">
+        <is>
+          <t>Multi Index FoF</t>
+        </is>
       </c>
       <c r="F796" t="n">
         <v>0</v>
@@ -30331,8 +30507,10 @@
       <c r="D797" t="n">
         <v>0</v>
       </c>
-      <c r="E797" t="n">
-        <v>0</v>
+      <c r="E797" t="inlineStr">
+        <is>
+          <t>Silver FoF</t>
+        </is>
       </c>
       <c r="F797" t="n">
         <v>0</v>
@@ -30365,8 +30543,10 @@
       <c r="D798" t="n">
         <v>0</v>
       </c>
-      <c r="E798" t="n">
-        <v>0</v>
+      <c r="E798" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F798" t="n">
         <v>0</v>
@@ -30399,8 +30579,10 @@
       <c r="D799" t="n">
         <v>0</v>
       </c>
-      <c r="E799" t="n">
-        <v>0</v>
+      <c r="E799" t="inlineStr">
+        <is>
+          <t>Other Competitor Thematic/Contra Funds</t>
+        </is>
       </c>
       <c r="F799" t="n">
         <v>0</v>
@@ -30433,8 +30615,10 @@
       <c r="D800" t="n">
         <v>0</v>
       </c>
-      <c r="E800" t="n">
-        <v>0</v>
+      <c r="E800" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F800" t="n">
         <v>0</v>
@@ -30467,8 +30651,10 @@
       <c r="D801" t="n">
         <v>0</v>
       </c>
-      <c r="E801" t="n">
-        <v>0</v>
+      <c r="E801" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F801" t="n">
         <v>0</v>
@@ -30501,8 +30687,10 @@
       <c r="D802" t="n">
         <v>0</v>
       </c>
-      <c r="E802" t="n">
-        <v>0</v>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F802" t="n">
         <v>0</v>
@@ -30535,8 +30723,10 @@
       <c r="D803" t="n">
         <v>0</v>
       </c>
-      <c r="E803" t="n">
-        <v>0</v>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>Pure International Plan</t>
+        </is>
       </c>
       <c r="F803" t="n">
         <v>0</v>
@@ -30569,8 +30759,10 @@
       <c r="D804" t="n">
         <v>0</v>
       </c>
-      <c r="E804" t="n">
-        <v>0</v>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F804" t="n">
         <v>0</v>
@@ -30603,8 +30795,10 @@
       <c r="D805" t="n">
         <v>0</v>
       </c>
-      <c r="E805" t="n">
-        <v>0</v>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F805" t="n">
         <v>0</v>
@@ -30637,8 +30831,10 @@
       <c r="D806" t="n">
         <v>0</v>
       </c>
-      <c r="E806" t="n">
-        <v>0</v>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F806" t="n">
         <v>0</v>
@@ -30671,8 +30867,10 @@
       <c r="D807" t="n">
         <v>0</v>
       </c>
-      <c r="E807" t="n">
-        <v>0</v>
+      <c r="E807" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F807" t="n">
         <v>0</v>
@@ -30705,8 +30903,10 @@
       <c r="D808" t="n">
         <v>0</v>
       </c>
-      <c r="E808" t="n">
-        <v>0</v>
+      <c r="E808" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F808" t="n">
         <v>0</v>
@@ -30739,8 +30939,10 @@
       <c r="D809" t="n">
         <v>0</v>
       </c>
-      <c r="E809" t="n">
-        <v>0</v>
+      <c r="E809" t="inlineStr">
+        <is>
+          <t>Asset Allocator Funds</t>
+        </is>
       </c>
       <c r="F809" t="n">
         <v>0</v>
@@ -30773,8 +30975,10 @@
       <c r="D810" t="n">
         <v>0</v>
       </c>
-      <c r="E810" t="n">
-        <v>0</v>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>Silver FoF</t>
+        </is>
       </c>
       <c r="F810" t="n">
         <v>0</v>
@@ -30807,8 +31011,10 @@
       <c r="D811" t="n">
         <v>0</v>
       </c>
-      <c r="E811" t="n">
-        <v>0</v>
+      <c r="E811" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 FOFs</t>
+        </is>
       </c>
       <c r="F811" t="n">
         <v>0</v>
@@ -30841,8 +31047,10 @@
       <c r="D812" t="n">
         <v>0</v>
       </c>
-      <c r="E812" t="n">
-        <v>0</v>
+      <c r="E812" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F812" t="n">
         <v>0</v>
@@ -30875,8 +31083,10 @@
       <c r="D813" t="n">
         <v>0</v>
       </c>
-      <c r="E813" t="n">
-        <v>0</v>
+      <c r="E813" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F813" t="n">
         <v>0</v>
@@ -30909,8 +31119,10 @@
       <c r="D814" t="n">
         <v>0</v>
       </c>
-      <c r="E814" t="n">
-        <v>0</v>
+      <c r="E814" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F814" t="n">
         <v>0</v>
@@ -30943,8 +31155,10 @@
       <c r="D815" t="n">
         <v>0</v>
       </c>
-      <c r="E815" t="n">
-        <v>0</v>
+      <c r="E815" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F815" t="n">
         <v>0</v>
@@ -30977,8 +31191,10 @@
       <c r="D816" t="n">
         <v>0</v>
       </c>
-      <c r="E816" t="n">
-        <v>0</v>
+      <c r="E816" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F816" t="n">
         <v>0</v>
@@ -31011,8 +31227,10 @@
       <c r="D817" t="n">
         <v>0</v>
       </c>
-      <c r="E817" t="n">
-        <v>0</v>
+      <c r="E817" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F817" t="n">
         <v>0</v>
@@ -31045,8 +31263,10 @@
       <c r="D818" t="n">
         <v>0</v>
       </c>
-      <c r="E818" t="n">
-        <v>0</v>
+      <c r="E818" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F818" t="n">
         <v>0</v>
@@ -31079,8 +31299,10 @@
       <c r="D819" t="n">
         <v>0</v>
       </c>
-      <c r="E819" t="n">
-        <v>0</v>
+      <c r="E819" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F819" t="n">
         <v>0</v>
@@ -31113,8 +31335,10 @@
       <c r="D820" t="n">
         <v>0</v>
       </c>
-      <c r="E820" t="n">
-        <v>0</v>
+      <c r="E820" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F820" t="n">
         <v>0</v>
@@ -31147,8 +31371,10 @@
       <c r="D821" t="n">
         <v>0</v>
       </c>
-      <c r="E821" t="n">
-        <v>0</v>
+      <c r="E821" t="inlineStr">
+        <is>
+          <t>Other Competitor Thematic/Contra Funds</t>
+        </is>
       </c>
       <c r="F821" t="n">
         <v>0</v>
@@ -31181,8 +31407,10 @@
       <c r="D822" t="n">
         <v>0</v>
       </c>
-      <c r="E822" t="n">
-        <v>0</v>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F822" t="n">
         <v>0</v>
@@ -31215,8 +31443,10 @@
       <c r="D823" t="n">
         <v>0</v>
       </c>
-      <c r="E823" t="n">
-        <v>0</v>
+      <c r="E823" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F823" t="n">
         <v>0</v>
@@ -31249,8 +31479,10 @@
       <c r="D824" t="n">
         <v>0</v>
       </c>
-      <c r="E824" t="n">
-        <v>0</v>
+      <c r="E824" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F824" t="n">
         <v>0</v>
@@ -31283,8 +31515,10 @@
       <c r="D825" t="n">
         <v>0</v>
       </c>
-      <c r="E825" t="n">
-        <v>0</v>
+      <c r="E825" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F825" t="n">
         <v>0</v>
@@ -31317,8 +31551,10 @@
       <c r="D826" t="n">
         <v>0</v>
       </c>
-      <c r="E826" t="n">
-        <v>0</v>
+      <c r="E826" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F826" t="n">
         <v>0</v>
@@ -31351,8 +31587,10 @@
       <c r="D827" t="n">
         <v>0</v>
       </c>
-      <c r="E827" t="n">
-        <v>0</v>
+      <c r="E827" t="inlineStr">
+        <is>
+          <t>Asset Allocator Funds</t>
+        </is>
       </c>
       <c r="F827" t="n">
         <v>0</v>
@@ -31385,8 +31623,10 @@
       <c r="D828" t="n">
         <v>0</v>
       </c>
-      <c r="E828" t="n">
-        <v>0</v>
+      <c r="E828" t="inlineStr">
+        <is>
+          <t>Asset Allocator Funds</t>
+        </is>
       </c>
       <c r="F828" t="n">
         <v>0</v>
@@ -31419,8 +31659,10 @@
       <c r="D829" t="n">
         <v>0</v>
       </c>
-      <c r="E829" t="n">
-        <v>0</v>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F829" t="n">
         <v>0</v>
@@ -31453,8 +31695,10 @@
       <c r="D830" t="n">
         <v>0</v>
       </c>
-      <c r="E830" t="n">
-        <v>0</v>
+      <c r="E830" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F830" t="n">
         <v>0</v>
@@ -31487,8 +31731,10 @@
       <c r="D831" t="n">
         <v>0</v>
       </c>
-      <c r="E831" t="n">
-        <v>0</v>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 FOFs</t>
+        </is>
       </c>
       <c r="F831" t="n">
         <v>0</v>
@@ -31521,8 +31767,10 @@
       <c r="D832" t="n">
         <v>0</v>
       </c>
-      <c r="E832" t="n">
-        <v>0</v>
+      <c r="E832" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F832" t="n">
         <v>0</v>
@@ -31555,8 +31803,10 @@
       <c r="D833" t="n">
         <v>0</v>
       </c>
-      <c r="E833" t="n">
-        <v>0</v>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F833" t="n">
         <v>0</v>
@@ -31589,8 +31839,10 @@
       <c r="D834" t="n">
         <v>0</v>
       </c>
-      <c r="E834" t="n">
-        <v>0</v>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F834" t="n">
         <v>0</v>
@@ -31623,8 +31875,10 @@
       <c r="D835" t="n">
         <v>0</v>
       </c>
-      <c r="E835" t="n">
-        <v>0</v>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F835" t="n">
         <v>0</v>
@@ -31657,8 +31911,10 @@
       <c r="D836" t="n">
         <v>0</v>
       </c>
-      <c r="E836" t="n">
-        <v>0</v>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>Asset Allocator Funds</t>
+        </is>
       </c>
       <c r="F836" t="n">
         <v>0</v>
@@ -31691,8 +31947,10 @@
       <c r="D837" t="n">
         <v>0</v>
       </c>
-      <c r="E837" t="n">
-        <v>0</v>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F837" t="n">
         <v>0</v>
@@ -31725,8 +31983,10 @@
       <c r="D838" t="n">
         <v>0</v>
       </c>
-      <c r="E838" t="n">
-        <v>0</v>
+      <c r="E838" t="inlineStr">
+        <is>
+          <t>Silver FoF</t>
+        </is>
       </c>
       <c r="F838" t="n">
         <v>0</v>
@@ -31759,8 +32019,10 @@
       <c r="D839" t="n">
         <v>0</v>
       </c>
-      <c r="E839" t="n">
-        <v>0</v>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>Pure International Plan</t>
+        </is>
       </c>
       <c r="F839" t="n">
         <v>0</v>
@@ -31793,8 +32055,10 @@
       <c r="D840" t="n">
         <v>0</v>
       </c>
-      <c r="E840" t="n">
-        <v>0</v>
+      <c r="E840" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F840" t="n">
         <v>0</v>
@@ -31827,8 +32091,10 @@
       <c r="D841" t="n">
         <v>0</v>
       </c>
-      <c r="E841" t="n">
-        <v>0</v>
+      <c r="E841" t="inlineStr">
+        <is>
+          <t>FoF Overseas</t>
+        </is>
       </c>
       <c r="F841" t="n">
         <v>0</v>
@@ -31861,8 +32127,10 @@
       <c r="D842" t="n">
         <v>0</v>
       </c>
-      <c r="E842" t="n">
-        <v>0</v>
+      <c r="E842" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F842" t="n">
         <v>0</v>
@@ -31895,8 +32163,10 @@
       <c r="D843" t="n">
         <v>0</v>
       </c>
-      <c r="E843" t="n">
-        <v>0</v>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F843" t="n">
         <v>0</v>
@@ -31929,8 +32199,10 @@
       <c r="D844" t="n">
         <v>0</v>
       </c>
-      <c r="E844" t="n">
-        <v>0</v>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F844" t="n">
         <v>0</v>
@@ -31963,8 +32235,10 @@
       <c r="D845" t="n">
         <v>0</v>
       </c>
-      <c r="E845" t="n">
-        <v>0</v>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F845" t="n">
         <v>0</v>
@@ -31997,8 +32271,10 @@
       <c r="D846" t="n">
         <v>0</v>
       </c>
-      <c r="E846" t="n">
-        <v>0</v>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F846" t="n">
         <v>0</v>
@@ -32031,8 +32307,10 @@
       <c r="D847" t="n">
         <v>0</v>
       </c>
-      <c r="E847" t="n">
-        <v>0</v>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F847" t="n">
         <v>0</v>
@@ -32065,8 +32343,10 @@
       <c r="D848" t="n">
         <v>0</v>
       </c>
-      <c r="E848" t="n">
-        <v>0</v>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F848" t="n">
         <v>0</v>
@@ -32099,8 +32379,10 @@
       <c r="D849" t="n">
         <v>0</v>
       </c>
-      <c r="E849" t="n">
-        <v>0</v>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F849" t="n">
         <v>0</v>
@@ -32133,8 +32415,10 @@
       <c r="D850" t="n">
         <v>0</v>
       </c>
-      <c r="E850" t="n">
-        <v>0</v>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>Pure International Plan</t>
+        </is>
       </c>
       <c r="F850" t="n">
         <v>0</v>
@@ -32167,8 +32451,10 @@
       <c r="D851" t="n">
         <v>0</v>
       </c>
-      <c r="E851" t="n">
-        <v>0</v>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F851" t="n">
         <v>0</v>
@@ -32201,8 +32487,10 @@
       <c r="D852" t="n">
         <v>0</v>
       </c>
-      <c r="E852" t="n">
-        <v>0</v>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F852" t="n">
         <v>0</v>
@@ -32235,8 +32523,10 @@
       <c r="D853" t="n">
         <v>0</v>
       </c>
-      <c r="E853" t="n">
-        <v>0</v>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F853" t="n">
         <v>0</v>
@@ -32269,8 +32559,10 @@
       <c r="D854" t="n">
         <v>0</v>
       </c>
-      <c r="E854" t="n">
-        <v>0</v>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F854" t="n">
         <v>0</v>
@@ -32303,8 +32595,10 @@
       <c r="D855" t="n">
         <v>0</v>
       </c>
-      <c r="E855" t="n">
-        <v>0</v>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F855" t="n">
         <v>0</v>
@@ -32337,8 +32631,10 @@
       <c r="D856" t="n">
         <v>0</v>
       </c>
-      <c r="E856" t="n">
-        <v>0</v>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F856" t="n">
         <v>0</v>
@@ -32371,8 +32667,10 @@
       <c r="D857" t="n">
         <v>0</v>
       </c>
-      <c r="E857" t="n">
-        <v>0</v>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F857" t="n">
         <v>0</v>
@@ -32405,8 +32703,10 @@
       <c r="D858" t="n">
         <v>0</v>
       </c>
-      <c r="E858" t="n">
-        <v>0</v>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F858" t="n">
         <v>0</v>
@@ -32439,8 +32739,10 @@
       <c r="D859" t="n">
         <v>0</v>
       </c>
-      <c r="E859" t="n">
-        <v>0</v>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F859" t="n">
         <v>0</v>
@@ -32473,8 +32775,10 @@
       <c r="D860" t="n">
         <v>0</v>
       </c>
-      <c r="E860" t="n">
-        <v>0</v>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>Silver FoF</t>
+        </is>
       </c>
       <c r="F860" t="n">
         <v>0</v>
@@ -32507,8 +32811,10 @@
       <c r="D861" t="n">
         <v>0</v>
       </c>
-      <c r="E861" t="n">
-        <v>0</v>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F861" t="n">
         <v>0</v>
@@ -32541,8 +32847,10 @@
       <c r="D862" t="n">
         <v>0</v>
       </c>
-      <c r="E862" t="n">
-        <v>0</v>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F862" t="n">
         <v>0</v>
@@ -32575,8 +32883,10 @@
       <c r="D863" t="n">
         <v>0</v>
       </c>
-      <c r="E863" t="n">
-        <v>0</v>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>FoF Domestic</t>
+        </is>
       </c>
       <c r="F863" t="n">
         <v>0</v>
@@ -32609,8 +32919,10 @@
       <c r="D864" t="n">
         <v>0</v>
       </c>
-      <c r="E864" t="n">
-        <v>0</v>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>Bal Bhavishya</t>
+        </is>
       </c>
       <c r="F864" t="n">
         <v>0</v>
@@ -32643,8 +32955,10 @@
       <c r="D865" t="n">
         <v>0</v>
       </c>
-      <c r="E865" t="n">
-        <v>0</v>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>Retirement Fund 30</t>
+        </is>
       </c>
       <c r="F865" t="n">
         <v>0</v>
@@ -32677,8 +32991,10 @@
       <c r="D866" t="n">
         <v>0</v>
       </c>
-      <c r="E866" t="n">
-        <v>0</v>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>Retirement Fund 40</t>
+        </is>
       </c>
       <c r="F866" t="n">
         <v>0</v>
@@ -32711,8 +33027,10 @@
       <c r="D867" t="n">
         <v>0</v>
       </c>
-      <c r="E867" t="n">
-        <v>0</v>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>Retirement Fund</t>
+        </is>
       </c>
       <c r="F867" t="n">
         <v>0</v>
@@ -32745,8 +33063,10 @@
       <c r="D868" t="n">
         <v>0</v>
       </c>
-      <c r="E868" t="n">
-        <v>0</v>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>Retirement Fund</t>
+        </is>
       </c>
       <c r="F868" t="n">
         <v>0</v>
@@ -32779,8 +33099,10 @@
       <c r="D869" t="n">
         <v>0</v>
       </c>
-      <c r="E869" t="n">
-        <v>0</v>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>Children's Fund</t>
+        </is>
       </c>
       <c r="F869" t="n">
         <v>0</v>
@@ -32813,8 +33135,10 @@
       <c r="D870" t="n">
         <v>0</v>
       </c>
-      <c r="E870" t="n">
-        <v>0</v>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>Retirement Fund 40</t>
+        </is>
       </c>
       <c r="F870" t="n">
         <v>0</v>
@@ -32847,8 +33171,10 @@
       <c r="D871" t="n">
         <v>0</v>
       </c>
-      <c r="E871" t="n">
-        <v>0</v>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>Retirement Fund</t>
+        </is>
       </c>
       <c r="F871" t="n">
         <v>0</v>
@@ -32881,8 +33207,10 @@
       <c r="D872" t="n">
         <v>0</v>
       </c>
-      <c r="E872" t="n">
-        <v>0</v>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>Retirement Fund 30</t>
+        </is>
       </c>
       <c r="F872" t="n">
         <v>0</v>
@@ -32915,8 +33243,10 @@
       <c r="D873" t="n">
         <v>0</v>
       </c>
-      <c r="E873" t="n">
-        <v>0</v>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>Retirement Fund</t>
+        </is>
       </c>
       <c r="F873" t="n">
         <v>0</v>
@@ -32949,8 +33279,10 @@
       <c r="D874" t="n">
         <v>0</v>
       </c>
-      <c r="E874" t="n">
-        <v>0</v>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>Children's Fund</t>
+        </is>
       </c>
       <c r="F874" t="n">
         <v>0</v>
@@ -32983,8 +33315,10 @@
       <c r="D875" t="n">
         <v>0</v>
       </c>
-      <c r="E875" t="n">
-        <v>0</v>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>Retirement Fund</t>
+        </is>
       </c>
       <c r="F875" t="n">
         <v>0</v>
@@ -33017,8 +33351,10 @@
       <c r="D876" t="n">
         <v>0</v>
       </c>
-      <c r="E876" t="n">
-        <v>0</v>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>Retirement Fund</t>
+        </is>
       </c>
       <c r="F876" t="n">
         <v>0</v>
@@ -33051,8 +33387,10 @@
       <c r="D877" t="n">
         <v>0</v>
       </c>
-      <c r="E877" t="n">
-        <v>0</v>
+      <c r="E877" t="inlineStr">
+        <is>
+          <t>Children's Fund</t>
+        </is>
       </c>
       <c r="F877" t="n">
         <v>0</v>
@@ -33085,8 +33423,10 @@
       <c r="D878" t="n">
         <v>0</v>
       </c>
-      <c r="E878" t="n">
-        <v>0</v>
+      <c r="E878" t="inlineStr">
+        <is>
+          <t>Retirement Fund 30</t>
+        </is>
       </c>
       <c r="F878" t="n">
         <v>0</v>
@@ -33119,8 +33459,10 @@
       <c r="D879" t="n">
         <v>0</v>
       </c>
-      <c r="E879" t="n">
-        <v>0</v>
+      <c r="E879" t="inlineStr">
+        <is>
+          <t>Retirement Fund</t>
+        </is>
       </c>
       <c r="F879" t="n">
         <v>0</v>
@@ -33153,8 +33495,10 @@
       <c r="D880" t="n">
         <v>0</v>
       </c>
-      <c r="E880" t="n">
-        <v>0</v>
+      <c r="E880" t="inlineStr">
+        <is>
+          <t>Retirement Fund 40</t>
+        </is>
       </c>
       <c r="F880" t="n">
         <v>0</v>
@@ -33187,8 +33531,10 @@
       <c r="D881" t="n">
         <v>0</v>
       </c>
-      <c r="E881" t="n">
-        <v>0</v>
+      <c r="E881" t="inlineStr">
+        <is>
+          <t>Children's Fund</t>
+        </is>
       </c>
       <c r="F881" t="n">
         <v>0</v>
@@ -33221,8 +33567,10 @@
       <c r="D882" t="n">
         <v>0</v>
       </c>
-      <c r="E882" t="n">
-        <v>0</v>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>Retirement Fund 40</t>
+        </is>
       </c>
       <c r="F882" t="n">
         <v>0</v>
@@ -33255,8 +33603,10 @@
       <c r="D883" t="n">
         <v>0</v>
       </c>
-      <c r="E883" t="n">
-        <v>0</v>
+      <c r="E883" t="inlineStr">
+        <is>
+          <t>Retirement Fund</t>
+        </is>
       </c>
       <c r="F883" t="n">
         <v>0</v>
@@ -33289,8 +33639,10 @@
       <c r="D884" t="n">
         <v>0</v>
       </c>
-      <c r="E884" t="n">
-        <v>0</v>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>Retirement Fund</t>
+        </is>
       </c>
       <c r="F884" t="n">
         <v>0</v>
@@ -33323,8 +33675,10 @@
       <c r="D885" t="n">
         <v>0</v>
       </c>
-      <c r="E885" t="n">
-        <v>0</v>
+      <c r="E885" t="inlineStr">
+        <is>
+          <t>Retirement Fund 30</t>
+        </is>
       </c>
       <c r="F885" t="n">
         <v>0</v>
@@ -33357,8 +33711,10 @@
       <c r="D886" t="n">
         <v>0</v>
       </c>
-      <c r="E886" t="n">
-        <v>0</v>
+      <c r="E886" t="inlineStr">
+        <is>
+          <t>Children's Fund</t>
+        </is>
       </c>
       <c r="F886" t="n">
         <v>0</v>
@@ -33391,8 +33747,10 @@
       <c r="D887" t="n">
         <v>0</v>
       </c>
-      <c r="E887" t="n">
-        <v>0</v>
+      <c r="E887" t="inlineStr">
+        <is>
+          <t>Retirement Fund</t>
+        </is>
       </c>
       <c r="F887" t="n">
         <v>0</v>
@@ -33425,8 +33783,10 @@
       <c r="D888" t="n">
         <v>0</v>
       </c>
-      <c r="E888" t="n">
-        <v>0</v>
+      <c r="E888" t="inlineStr">
+        <is>
+          <t>Retirement Fund 30</t>
+        </is>
       </c>
       <c r="F888" t="n">
         <v>0</v>
@@ -33459,8 +33819,10 @@
       <c r="D889" t="n">
         <v>0</v>
       </c>
-      <c r="E889" t="n">
-        <v>0</v>
+      <c r="E889" t="inlineStr">
+        <is>
+          <t>Retirement Fund 30</t>
+        </is>
       </c>
       <c r="F889" t="n">
         <v>0</v>
@@ -33493,8 +33855,10 @@
       <c r="D890" t="n">
         <v>0</v>
       </c>
-      <c r="E890" t="n">
-        <v>0</v>
+      <c r="E890" t="inlineStr">
+        <is>
+          <t>Children's Fund</t>
+        </is>
       </c>
       <c r="F890" t="n">
         <v>0</v>
@@ -33527,8 +33891,10 @@
       <c r="D891" t="n">
         <v>0</v>
       </c>
-      <c r="E891" t="n">
-        <v>0</v>
+      <c r="E891" t="inlineStr">
+        <is>
+          <t>Children's Fund</t>
+        </is>
       </c>
       <c r="F891" t="n">
         <v>0</v>
@@ -33561,8 +33927,10 @@
       <c r="D892" t="n">
         <v>0</v>
       </c>
-      <c r="E892" t="n">
-        <v>0</v>
+      <c r="E892" t="inlineStr">
+        <is>
+          <t>Retirement Fund 40</t>
+        </is>
       </c>
       <c r="F892" t="n">
         <v>0</v>
@@ -33595,8 +33963,10 @@
       <c r="D893" t="n">
         <v>0</v>
       </c>
-      <c r="E893" t="n">
-        <v>0</v>
+      <c r="E893" t="inlineStr">
+        <is>
+          <t>Retirement Fund 30</t>
+        </is>
       </c>
       <c r="F893" t="n">
         <v>0</v>
@@ -33629,8 +33999,10 @@
       <c r="D894" t="n">
         <v>0</v>
       </c>
-      <c r="E894" t="n">
-        <v>0</v>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>Retirement Fund</t>
+        </is>
       </c>
       <c r="F894" t="n">
         <v>0</v>
@@ -33663,8 +34035,10 @@
       <c r="D895" t="n">
         <v>0</v>
       </c>
-      <c r="E895" t="n">
-        <v>0</v>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>Retirement Fund</t>
+        </is>
       </c>
       <c r="F895" t="n">
         <v>0</v>
@@ -33697,8 +34071,10 @@
       <c r="D896" t="n">
         <v>0</v>
       </c>
-      <c r="E896" t="n">
-        <v>0</v>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>Bal Bhavishya</t>
+        </is>
       </c>
       <c r="F896" t="n">
         <v>0</v>
@@ -33731,8 +34107,10 @@
       <c r="D897" t="n">
         <v>0</v>
       </c>
-      <c r="E897" t="n">
-        <v>0</v>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>Retirement Fund 40</t>
+        </is>
       </c>
       <c r="F897" t="n">
         <v>0</v>
@@ -33765,8 +34143,10 @@
       <c r="D898" t="n">
         <v>0</v>
       </c>
-      <c r="E898" t="n">
-        <v>0</v>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>Retirement Fund</t>
+        </is>
       </c>
       <c r="F898" t="n">
         <v>0</v>
@@ -33799,8 +34179,10 @@
       <c r="D899" t="n">
         <v>0</v>
       </c>
-      <c r="E899" t="n">
-        <v>0</v>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>Retirement Fund 30</t>
+        </is>
       </c>
       <c r="F899" t="n">
         <v>0</v>
@@ -33833,8 +34215,10 @@
       <c r="D900" t="n">
         <v>0</v>
       </c>
-      <c r="E900" t="n">
-        <v>0</v>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>Children's Fund</t>
+        </is>
       </c>
       <c r="F900" t="n">
         <v>0</v>
@@ -33867,8 +34251,10 @@
       <c r="D901" t="n">
         <v>0</v>
       </c>
-      <c r="E901" t="n">
-        <v>0</v>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>Retirement Fund 30</t>
+        </is>
       </c>
       <c r="F901" t="n">
         <v>0</v>
@@ -33901,8 +34287,10 @@
       <c r="D902" t="n">
         <v>0</v>
       </c>
-      <c r="E902" t="n">
-        <v>0</v>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>Bal Bhavishya</t>
+        </is>
       </c>
       <c r="F902" t="n">
         <v>0</v>
@@ -33935,8 +34323,10 @@
       <c r="D903" t="n">
         <v>0</v>
       </c>
-      <c r="E903" t="n">
-        <v>0</v>
+      <c r="E903" t="inlineStr">
+        <is>
+          <t>Children's Fund</t>
+        </is>
       </c>
       <c r="F903" t="n">
         <v>0</v>
@@ -33969,8 +34359,10 @@
       <c r="D904" t="n">
         <v>0</v>
       </c>
-      <c r="E904" t="n">
-        <v>0</v>
+      <c r="E904" t="inlineStr">
+        <is>
+          <t>Retirement Fund</t>
+        </is>
       </c>
       <c r="F904" t="n">
         <v>0</v>
@@ -35751,8 +36143,10 @@
       <c r="D951" t="n">
         <v>0</v>
       </c>
-      <c r="E951" t="n">
-        <v>0</v>
+      <c r="E951" t="inlineStr">
+        <is>
+          <t>Children's Fund</t>
+        </is>
       </c>
       <c r="F951" t="n">
         <v>0</v>
@@ -35765,6 +36159,114 @@
       <c r="H951" t="inlineStr">
         <is>
           <t>Axis Childrens Fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="n">
+        <v>149291</v>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>Aditya Birla Sun Life US Equity Passive FOF - Dir - Growth</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D952" t="n">
+        <v>0</v>
+      </c>
+      <c r="E952" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 FOFs</t>
+        </is>
+      </c>
+      <c r="F952" t="n">
+        <v>0</v>
+      </c>
+      <c r="G952" t="inlineStr">
+        <is>
+          <t>BIR1219</t>
+        </is>
+      </c>
+      <c r="H952" t="inlineStr">
+        <is>
+          <t>Aditya Birla Sun Life US Equity Passive FOF</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="n">
+        <v>150751</v>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>Axis NASDAQ 100 US Specific Equity Passive FOF - Dir - Growth</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D953" t="n">
+        <v>0</v>
+      </c>
+      <c r="E953" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 FOFs</t>
+        </is>
+      </c>
+      <c r="F953" t="n">
+        <v>0</v>
+      </c>
+      <c r="G953" t="inlineStr">
+        <is>
+          <t>AXI0387</t>
+        </is>
+      </c>
+      <c r="H953" t="inlineStr">
+        <is>
+          <t>Axis NASDAQ 100 US Specific Equity Passive FOF</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="n">
+        <v>145552</v>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>Motilal Oswal Nasdaq 100 FOF - Dir - Growth</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D954" t="n">
+        <v>0</v>
+      </c>
+      <c r="E954" t="inlineStr">
+        <is>
+          <t>Nasdaq 100 FOFs</t>
+        </is>
+      </c>
+      <c r="F954" t="n">
+        <v>0</v>
+      </c>
+      <c r="G954" t="inlineStr">
+        <is>
+          <t>MOT0015</t>
+        </is>
+      </c>
+      <c r="H954" t="inlineStr">
+        <is>
+          <t>Motilal Oswal Nasdaq 100 Fund of Fund</t>
         </is>
       </c>
     </row>

</xml_diff>